<commit_message>
Restore coat-of-arms logo on Luiza MCF inventory sheets
The previous build dropped the embedded header logo because Pillow was
not available at save time. Rebuilt with Pillow so the armoiries banner
is preserved on all three sheets (same anchor/design as the model).
</commit_message>
<xml_diff>
--- a/INVENTAIRE_DES_MCF_ANTENNE_PEV_LUIZA_FEVRIER_2026_VF.xlsx
+++ b/INVENTAIRE_DES_MCF_ANTENNE_PEV_LUIZA_FEVRIER_2026_VF.xlsx
@@ -1139,6 +1139,150 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <twoCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>1</rowOff>
+    </from>
+    <to>
+      <col>3</col>
+      <colOff>971550</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 25" descr="wps1"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="1"/>
+          <a:ext cx="6172200" cy="1466850"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <twoCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>1</rowOff>
+    </from>
+    <to>
+      <col>4</col>
+      <colOff>971550</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 25" descr="wps1"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="1"/>
+          <a:ext cx="6172200" cy="1333499"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <twoCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>247650</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <to>
+      <col>4</col>
+      <colOff>133350</colOff>
+      <row>6</row>
+      <rowOff>190499</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 25" descr="wps1"/>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="247650" y="0"/>
+          <a:ext cx="6781800" cy="1333499"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
@@ -7140,6 +7284,7 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -7895,6 +8040,7 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" scale="68"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -8271,5 +8417,6 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" scale="93"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>